<commit_message>
Start crypto plan on 10 Feb 2027 with buys on the 10th of each month
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CGfptAUVN8T4prJmapx7Bb
</commit_message>
<xml_diff>
--- a/crypto_plan_1lakh_2027_2028.xlsx
+++ b/crypto_plan_1lakh_2027_2028.xlsx
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="185">
   <si>
     <t xml:space="preserve">Crypto Plan 2027–2028 — Inputs</t>
   </si>
@@ -160,7 +160,7 @@
     <t xml:space="preserve">Number of monthly buys</t>
   </si>
   <si>
-    <t xml:space="preserve">Jan–Dec 2027.</t>
+    <t xml:space="preserve">On the 10th of each month, 10 Feb 2027 – 10 Jan 2028.</t>
   </si>
   <si>
     <t xml:space="preserve">Tax on crypto gains</t>
@@ -256,7 +256,7 @@
     <t xml:space="preserve">Buy Plan — how much to buy, and at which price</t>
   </si>
   <si>
-    <t xml:space="preserve">Monthly buy on the 1st of each month in 2027. Dip orders = limit orders; if not filled by Jul 2028, buy at market that month.</t>
+    <t xml:space="preserve">Monthly buy on the 10th of each month, 10 Feb 2027 – 10 Jan 2028. Dip orders = limit orders; if not filled by Jul 2028, buy at market that month.</t>
   </si>
   <si>
     <t xml:space="preserve">Total for coin (₹)</t>
@@ -304,13 +304,13 @@
     <t xml:space="preserve">Indian exchanges quote INR prices: compare the USD price on the exchange's USDT market, or adjust the ₹ levels for the exchange premium.</t>
   </si>
   <si>
-    <t xml:space="preserve">Month-by-month plan, Jan 2027 – Dec 2028</t>
+    <t xml:space="preserve">Month-by-month plan, 10 Feb 2027 – Dec 2028</t>
   </si>
   <si>
     <t xml:space="preserve">Buy amounts update from 'Buy Plan'. 'Past cycles' = BTC's average return in the matching month of the 2017–21 and 2021–25 cycles (guide only).</t>
   </si>
   <si>
-    <t xml:space="preserve">Month</t>
+    <t xml:space="preserve">Month (buy on 10th)</t>
   </si>
   <si>
     <t xml:space="preserve">Past cycles (BTC avg)</t>
@@ -355,67 +355,61 @@
     <t xml:space="preserve">Done? (✓)</t>
   </si>
   <si>
-    <t xml:space="preserve">Jan 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monthly buy. Place Dip 1 and Dip 2 limit orders for every coin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feb 2027</t>
+    <t xml:space="preserve">10 Feb 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">START 10 Feb 2027: first monthly buy. Place Dip 1 and Dip 2 limit orders for every coin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Mar 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly buy (prices often jump here — don't chase).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Apr 2027</t>
   </si>
   <si>
     <t xml:space="preserve">Monthly buy.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mar 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monthly buy (prices often jump here — don't chase).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apr 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 2027</t>
+    <t xml:space="preserve">10 May 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Jun 2027</t>
   </si>
   <si>
     <t xml:space="preserve">Monthly buy. Watch for dip orders to fill.</t>
   </si>
   <si>
-    <t xml:space="preserve">Jul 2027</t>
+    <t xml:space="preserve">10 Jul 2027</t>
   </si>
   <si>
     <t xml:space="preserve">Monthly buy. Best month to buy in this pattern (fell in both cycles).</t>
   </si>
   <si>
-    <t xml:space="preserve">Aug 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sep 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oct 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nov 2027</t>
+    <t xml:space="preserve">10 Aug 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Sep 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Oct 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Nov 2027</t>
   </si>
   <si>
     <t xml:space="preserve">Monthly buy (often a strong month).</t>
   </si>
   <si>
-    <t xml:space="preserve">Dec 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last monthly buy. Check dip orders are still open.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jan 2028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No monthly buy. Keep dip orders open.</t>
+    <t xml:space="preserve">10 Dec 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 Jan 2028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last (12th) monthly buy on 10 Jan. Check dip orders are still open.</t>
   </si>
   <si>
     <t xml:space="preserve">Feb 2028</t>
@@ -559,7 +553,7 @@
     <t xml:space="preserve">Example (format only, not counted):</t>
   </si>
   <si>
-    <t xml:space="preserve">01-Jan-2027</t>
+    <t xml:space="preserve">10-Feb-2027</t>
   </si>
   <si>
     <t xml:space="preserve">Buy</t>
@@ -2219,7 +2213,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -2295,7 +2289,7 @@
         <v>78</v>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04</v>
+        <v>0.26</v>
       </c>
       <c r="C5" s="22" t="n">
         <v>1</v>
@@ -2349,7 +2343,7 @@
         <v>80</v>
       </c>
       <c r="B6" s="10" t="n">
-        <v>0.26</v>
+        <v>0.32</v>
       </c>
       <c r="C6" s="22" t="n">
         <v>1</v>
@@ -2403,7 +2397,7 @@
         <v>82</v>
       </c>
       <c r="B7" s="10" t="n">
-        <v>0.32</v>
+        <v>0.1</v>
       </c>
       <c r="C7" s="22" t="n">
         <v>1</v>
@@ -2457,7 +2451,7 @@
         <v>84</v>
       </c>
       <c r="B8" s="10" t="n">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="C8" s="22" t="n">
         <v>1</v>
@@ -2502,7 +2496,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O8" s="24"/>
     </row>
@@ -2511,7 +2505,7 @@
         <v>85</v>
       </c>
       <c r="B9" s="10" t="n">
-        <v>0.02</v>
+        <v>-0.04</v>
       </c>
       <c r="C9" s="22" t="n">
         <v>1</v>
@@ -2556,16 +2550,16 @@
         <v>0</v>
       </c>
       <c r="N9" s="23" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="O9" s="24"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B10" s="10" t="n">
-        <v>-0.04</v>
+        <v>-0.12</v>
       </c>
       <c r="C10" s="22" t="n">
         <v>1</v>
@@ -2610,16 +2604,16 @@
         <v>0</v>
       </c>
       <c r="N10" s="23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O10" s="24"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B11" s="10" t="n">
-        <v>-0.12</v>
+        <v>0.07</v>
       </c>
       <c r="C11" s="22" t="n">
         <v>1</v>
@@ -2664,7 +2658,7 @@
         <v>0</v>
       </c>
       <c r="N11" s="23" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="O11" s="24"/>
     </row>
@@ -2673,7 +2667,7 @@
         <v>90</v>
       </c>
       <c r="B12" s="10" t="n">
-        <v>0.07</v>
+        <v>0.05</v>
       </c>
       <c r="C12" s="22" t="n">
         <v>1</v>
@@ -2718,7 +2712,7 @@
         <v>0</v>
       </c>
       <c r="N12" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O12" s="24"/>
     </row>
@@ -2727,7 +2721,7 @@
         <v>91</v>
       </c>
       <c r="B13" s="10" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="C13" s="22" t="n">
         <v>1</v>
@@ -2772,7 +2766,7 @@
         <v>0</v>
       </c>
       <c r="N13" s="23" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="O13" s="24"/>
     </row>
@@ -2781,7 +2775,7 @@
         <v>92</v>
       </c>
       <c r="B14" s="10" t="n">
-        <v>0.02</v>
+        <v>0.21</v>
       </c>
       <c r="C14" s="22" t="n">
         <v>1</v>
@@ -2826,16 +2820,16 @@
         <v>0</v>
       </c>
       <c r="N14" s="23" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="O14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B15" s="10" t="n">
-        <v>0.21</v>
+        <v>-0.04</v>
       </c>
       <c r="C15" s="22" t="n">
         <v>1</v>
@@ -2880,7 +2874,7 @@
         <v>0</v>
       </c>
       <c r="N15" s="23" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="O15" s="24"/>
     </row>
@@ -2889,7 +2883,7 @@
         <v>95</v>
       </c>
       <c r="B16" s="10" t="n">
-        <v>-0.04</v>
+        <v>0.09</v>
       </c>
       <c r="C16" s="22" t="n">
         <v>1</v>
@@ -2943,7 +2937,7 @@
         <v>97</v>
       </c>
       <c r="B17" s="10" t="n">
-        <v>0.09</v>
+        <v>0.26</v>
       </c>
       <c r="C17" s="22" t="n">
         <v>0</v>
@@ -2993,11 +2987,11 @@
       <c r="O17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="25" t="s">
         <v>99</v>
       </c>
       <c r="B18" s="10" t="n">
-        <v>0.26</v>
+        <v>-0.03</v>
       </c>
       <c r="C18" s="22" t="n">
         <v>0</v>
@@ -3039,19 +3033,19 @@
         <v>60000</v>
       </c>
       <c r="M18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="14" t="s">
+        <v>0.1</v>
+      </c>
+      <c r="N18" s="26" t="s">
         <v>100</v>
       </c>
       <c r="O18" s="24"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="3" t="s">
         <v>101</v>
       </c>
       <c r="B19" s="10" t="n">
-        <v>-0.03</v>
+        <v>0.04</v>
       </c>
       <c r="C19" s="22" t="n">
         <v>0</v>
@@ -3093,9 +3087,9 @@
         <v>60000</v>
       </c>
       <c r="M19" s="10" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="N19" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="N19" s="14" t="s">
         <v>102</v>
       </c>
       <c r="O19" s="24"/>
@@ -3105,7 +3099,7 @@
         <v>103</v>
       </c>
       <c r="B20" s="10" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="C20" s="22" t="n">
         <v>0</v>
@@ -3150,16 +3144,16 @@
         <v>0</v>
       </c>
       <c r="N20" s="14" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="O20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B21" s="10" t="n">
-        <v>0.08</v>
+        <v>0.03</v>
       </c>
       <c r="C21" s="22" t="n">
         <v>0</v>
@@ -3204,16 +3198,16 @@
         <v>0</v>
       </c>
       <c r="N21" s="14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="O21" s="24"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B22" s="10" t="n">
-        <v>0.03</v>
+        <v>-0.08</v>
       </c>
       <c r="C22" s="22" t="n">
         <v>0</v>
@@ -3258,7 +3252,7 @@
         <v>0</v>
       </c>
       <c r="N22" s="14" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="O22" s="24"/>
     </row>
@@ -3267,7 +3261,7 @@
         <v>107</v>
       </c>
       <c r="B23" s="10" t="n">
-        <v>-0.08</v>
+        <v>0.18</v>
       </c>
       <c r="C23" s="22" t="n">
         <v>0</v>
@@ -3317,11 +3311,11 @@
       <c r="O23" s="24"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="25" t="s">
         <v>109</v>
       </c>
       <c r="B24" s="10" t="n">
-        <v>0.18</v>
+        <v>0.27</v>
       </c>
       <c r="C24" s="22" t="n">
         <v>0</v>
@@ -3363,9 +3357,9 @@
         <v>60000</v>
       </c>
       <c r="M24" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="14" t="s">
+        <v>0.1</v>
+      </c>
+      <c r="N24" s="26" t="s">
         <v>110</v>
       </c>
       <c r="O24" s="24"/>
@@ -3375,7 +3369,7 @@
         <v>111</v>
       </c>
       <c r="B25" s="10" t="n">
-        <v>0.27</v>
+        <v>0.42</v>
       </c>
       <c r="C25" s="22" t="n">
         <v>0</v>
@@ -3417,7 +3411,7 @@
         <v>60000</v>
       </c>
       <c r="M25" s="10" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="N25" s="26" t="s">
         <v>112</v>
@@ -3429,7 +3423,7 @@
         <v>113</v>
       </c>
       <c r="B26" s="10" t="n">
-        <v>0.42</v>
+        <v>0.06</v>
       </c>
       <c r="C26" s="22" t="n">
         <v>0</v>
@@ -3471,7 +3465,7 @@
         <v>60000</v>
       </c>
       <c r="M26" s="10" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="N26" s="26" t="s">
         <v>114</v>
@@ -3483,7 +3477,7 @@
         <v>115</v>
       </c>
       <c r="B27" s="10" t="n">
-        <v>0.06</v>
+        <v>0.23</v>
       </c>
       <c r="C27" s="22" t="n">
         <v>0</v>
@@ -3525,7 +3519,7 @@
         <v>60000</v>
       </c>
       <c r="M27" s="10" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="N27" s="26" t="s">
         <v>116</v>
@@ -3533,117 +3527,63 @@
       <c r="O27" s="24"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D28" s="16" t="n">
+        <f aca="false">SUM(D5:D27)</f>
+        <v>27000</v>
+      </c>
+      <c r="E28" s="16" t="n">
+        <f aca="false">SUM(E5:E27)</f>
+        <v>9000</v>
+      </c>
+      <c r="F28" s="16" t="n">
+        <f aca="false">SUM(F5:F27)</f>
+        <v>9000</v>
+      </c>
+      <c r="G28" s="16" t="n">
+        <f aca="false">SUM(G5:G27)</f>
+        <v>6000</v>
+      </c>
+      <c r="H28" s="16" t="n">
+        <f aca="false">SUM(H5:H27)</f>
+        <v>3000</v>
+      </c>
+      <c r="I28" s="16" t="n">
+        <f aca="false">SUM(I5:I27)</f>
+        <v>3000</v>
+      </c>
+      <c r="J28" s="16" t="n">
+        <f aca="false">SUM(J5:J27)</f>
+        <v>3000</v>
+      </c>
+      <c r="K28" s="16" t="n">
+        <f aca="false">SUM(K5:K27)</f>
+        <v>60000</v>
+      </c>
+      <c r="M28" s="15" t="n">
+        <f aca="false">SUM(M5:M27)</f>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="B28" s="10" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="C28" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="11" t="n">
-        <f aca="false">$C28*'Buy Plan'!$C$5</f>
-        <v>0</v>
-      </c>
-      <c r="E28" s="11" t="n">
-        <f aca="false">$C28*'Buy Plan'!$C$6</f>
-        <v>0</v>
-      </c>
-      <c r="F28" s="11" t="n">
-        <f aca="false">$C28*'Buy Plan'!$C$7</f>
-        <v>0</v>
-      </c>
-      <c r="G28" s="11" t="n">
-        <f aca="false">$C28*'Buy Plan'!$C$8</f>
-        <v>0</v>
-      </c>
-      <c r="H28" s="11" t="n">
-        <f aca="false">$C28*'Buy Plan'!$C$9</f>
-        <v>0</v>
-      </c>
-      <c r="I28" s="11" t="n">
-        <f aca="false">$C28*'Buy Plan'!$C$10</f>
-        <v>0</v>
-      </c>
-      <c r="J28" s="11" t="n">
-        <f aca="false">$C28*'Buy Plan'!$C$11</f>
-        <v>0</v>
-      </c>
-      <c r="K28" s="11" t="n">
-        <f aca="false">SUM(D28:J28)</f>
-        <v>0</v>
-      </c>
-      <c r="L28" s="11" t="n">
-        <f aca="false">L27+K28</f>
-        <v>60000</v>
-      </c>
-      <c r="M28" s="10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N28" s="26" t="s">
-        <v>118</v>
-      </c>
-      <c r="O28" s="24"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D29" s="16" t="n">
-        <f aca="false">SUM(D5:D28)</f>
-        <v>27000</v>
-      </c>
-      <c r="E29" s="16" t="n">
-        <f aca="false">SUM(E5:E28)</f>
-        <v>9000</v>
-      </c>
-      <c r="F29" s="16" t="n">
-        <f aca="false">SUM(F5:F28)</f>
-        <v>9000</v>
-      </c>
-      <c r="G29" s="16" t="n">
-        <f aca="false">SUM(G5:G28)</f>
-        <v>6000</v>
-      </c>
-      <c r="H29" s="16" t="n">
-        <f aca="false">SUM(H5:H28)</f>
-        <v>3000</v>
-      </c>
-      <c r="I29" s="16" t="n">
-        <f aca="false">SUM(I5:I28)</f>
-        <v>3000</v>
-      </c>
-      <c r="J29" s="16" t="n">
-        <f aca="false">SUM(J5:J28)</f>
-        <v>3000</v>
-      </c>
-      <c r="K29" s="16" t="n">
-        <f aca="false">SUM(K5:K28)</f>
-        <v>60000</v>
-      </c>
-      <c r="M29" s="15" t="n">
-        <f aca="false">SUM(M5:M28)</f>
-        <v>0.6</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B5:B28">
+  <conditionalFormatting sqref="B5:B27">
     <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3684,12 +3624,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3697,43 +3637,43 @@
         <v>18</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="H4" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="I4" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="J4" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="K4" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="L4" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="K4" s="9" t="s">
+      <c r="M4" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="N4" s="9" t="s">
         <v>134</v>
-      </c>
-      <c r="M4" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="N4" s="9" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4109,75 +4049,75 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B18" s="30" t="n">
-        <f aca="false">INDEX('Monthly Schedule'!$M$5:$M$28,MATCH(A18,'Monthly Schedule'!$A$5:$A$28,0))</f>
+        <f aca="false">INDEX('Monthly Schedule'!$M$5:$M$27,MATCH(A18,'Monthly Schedule'!$A$5:$A$27,0))</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B19" s="30" t="n">
-        <f aca="false">INDEX('Monthly Schedule'!$M$5:$M$28,MATCH(A19,'Monthly Schedule'!$A$5:$A$28,0))</f>
+        <f aca="false">INDEX('Monthly Schedule'!$M$5:$M$27,MATCH(A19,'Monthly Schedule'!$A$5:$A$27,0))</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B20" s="30" t="n">
-        <f aca="false">INDEX('Monthly Schedule'!$M$5:$M$28,MATCH(A20,'Monthly Schedule'!$A$5:$A$28,0))</f>
+        <f aca="false">INDEX('Monthly Schedule'!$M$5:$M$27,MATCH(A20,'Monthly Schedule'!$A$5:$A$27,0))</f>
         <v>0.15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B21" s="30" t="n">
-        <f aca="false">INDEX('Monthly Schedule'!$M$5:$M$28,MATCH(A21,'Monthly Schedule'!$A$5:$A$28,0))</f>
+        <f aca="false">INDEX('Monthly Schedule'!$M$5:$M$27,MATCH(A21,'Monthly Schedule'!$A$5:$A$27,0))</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B22" s="30" t="n">
-        <f aca="false">INDEX('Monthly Schedule'!$M$5:$M$28,MATCH(A22,'Monthly Schedule'!$A$5:$A$28,0))</f>
+        <f aca="false">INDEX('Monthly Schedule'!$M$5:$M$27,MATCH(A22,'Monthly Schedule'!$A$5:$A$27,0))</f>
         <v>0.15</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B23" s="15" t="n">
         <f aca="false">SUM(B18:B22)</f>
@@ -4228,28 +4168,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="31" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="32" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B4" s="32" t="s">
         <v>27</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D4" s="33" t="n">
         <v>7800000</v>
@@ -4266,75 +4206,75 @@
         <v>0</v>
       </c>
       <c r="H4" s="32" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>20</v>
       </c>
       <c r="F6" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="H6" s="9" t="s">
         <v>152</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>154</v>
       </c>
       <c r="J6" s="9" t="s">
         <v>18</v>
       </c>
       <c r="K6" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="M6" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="L6" s="9" t="s">
+      <c r="N6" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="M6" s="9" t="s">
+      <c r="O6" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="N6" s="9" t="s">
+      <c r="P6" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="O6" s="9" t="s">
+      <c r="Q6" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="P6" s="9" t="s">
+      <c r="R6" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="Q6" s="9" t="s">
+      <c r="S6" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="R6" s="9" t="s">
+      <c r="T6" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="S6" s="9" t="s">
+      <c r="U6" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="T6" s="9" t="s">
+      <c r="V6" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="W6" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="U6" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="V6" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="W6" s="9" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4909,7 +4849,7 @@
       </c>
       <c r="H16" s="39"/>
       <c r="J16" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7995,27 +7935,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="42" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="43" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8023,22 +7963,22 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="42" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="43" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="43" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="43" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8046,22 +7986,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="42" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="43" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="43" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="43" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8069,32 +8009,32 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="42" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="43" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="43" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="43" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="43" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="43" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>